<commit_message>
chore: update filled test-case workbook from latest run
</commit_message>
<xml_diff>
--- a/reports/test-cases-filled.xlsx
+++ b/reports/test-cases-filled.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="590">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -249,6 +249,9 @@
     <t>Access is granted to all instance level functions</t>
   </si>
   <si>
+    <t>Automated check failed: Error: Sidebar entry "Users" should be available</t>
+  </si>
+  <si>
     <t xml:space="preserve">USER MANAGEMENT </t>
   </si>
   <si>
@@ -266,6 +269,9 @@
   </si>
   <si>
     <t>- List of users displayed.- Users show key attributes (name, email, role, country, status, association).</t>
+  </si>
+  <si>
+    <t>Automated check failed: Test timeout of 30000ms exceeded while running "beforeEach" hook.</t>
   </si>
   <si>
     <t>IA-FM01-F15-TC02</t>
@@ -302,9 +308,6 @@
     <t>- Only users from selected country are displayed.</t>
   </si>
   <si>
-    <t>Automated check failed: Error: No location/country filter control is present on the Users list</t>
-  </si>
-  <si>
     <t>IA-FM01-F15-TC04</t>
   </si>
   <si>
@@ -321,9 +324,6 @@
     <t>- Users displayed match selected role.</t>
   </si>
   <si>
-    <t>Automated check failed: Error: No role filter control is present on the Users list</t>
-  </si>
-  <si>
     <t>IA-FM01-F15-TC05</t>
   </si>
   <si>
@@ -337,9 +337,6 @@
   </si>
   <si>
     <t>- Only users with selected status are shown.</t>
-  </si>
-  <si>
-    <t>Automated check failed: Error: No status filter control is present on the Users list</t>
   </si>
   <si>
     <t>IA-FM01-F15-TC06</t>
@@ -572,9 +569,6 @@
   </si>
   <si>
     <t>Permission assigned</t>
-  </si>
-  <si>
-    <t>Automated check failed: Error: No permission-assignment UI is present in the role editor (only an Active toggle exists)</t>
   </si>
   <si>
     <t>IA-FM01-F03-TC09</t>
@@ -750,6 +744,9 @@
     <t xml:space="preserve"> level created successfully</t>
   </si>
   <si>
+    <t>Automated check failed: Error: expect(locator).toBeVisible() failed</t>
+  </si>
+  <si>
     <t>IA-FM01-F10-TC02</t>
   </si>
   <si>
@@ -854,9 +851,6 @@
     <t>Inactive not visible</t>
   </si>
   <si>
-    <t>Automated check failed: Error: Inactive level should not be visible in the default list</t>
-  </si>
-  <si>
     <t>IA-FM01-F10-TC09</t>
   </si>
   <si>
@@ -907,9 +901,6 @@
     <t>Location level not listed on options</t>
   </si>
   <si>
-    <t>Automated check failed: Error: Location form uses a free-text Level ID (no options list), so inactive-level exclusion cannot be enforced/verified here</t>
-  </si>
-  <si>
     <t>IA-FM01-F10-TC12</t>
   </si>
   <si>
@@ -999,9 +990,6 @@
     <t>All users exported</t>
   </si>
   <si>
-    <t>Automated check failed: Error: No export/download control is present on the Users list</t>
-  </si>
-  <si>
     <t>IA-FM01-F15-TC15</t>
   </si>
   <si>
@@ -1247,9 +1235,6 @@
   </si>
   <si>
     <t>- Only associations from selected country displayed.</t>
-  </si>
-  <si>
-    <t>Automated check failed: Error: No country/location filter control on the Associations list (only status tabs exist)</t>
   </si>
   <si>
     <t>IA-CM05-F01-TC04</t>
@@ -1716,9 +1701,6 @@
   </si>
   <si>
     <t>List of email templates displays</t>
-  </si>
-  <si>
-    <t>Automated check failed: Error: No Email/SMS template configuration section is exposed in the instance admin portal navigation</t>
   </si>
   <si>
     <t xml:space="preserve"> IA-FM01-F22-TC02</t>
@@ -2468,10 +2450,10 @@
         <v>45935</v>
       </c>
       <c r="O3" s="18">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P3" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -2516,10 +2498,10 @@
         <v>45935</v>
       </c>
       <c r="O4" s="18">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P4" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -2700,10 +2682,10 @@
       <c r="M8" s="5"/>
       <c r="N8" s="12"/>
       <c r="O8" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P8" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -2774,10 +2756,10 @@
         <v>45935</v>
       </c>
       <c r="O10" s="18">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P10" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -2822,10 +2804,10 @@
         <v>45935</v>
       </c>
       <c r="O11" s="18">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P11" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -2848,13 +2830,13 @@
         <v>35</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="J12" s="17">
         <v>45877</v>
@@ -2870,15 +2852,15 @@
         <v>45935</v>
       </c>
       <c r="O12" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P12" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -2900,31 +2882,31 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H14" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J14" s="17">
         <v>45877</v>
@@ -2940,39 +2922,39 @@
         <v>45935</v>
       </c>
       <c r="O14" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P14" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B15" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="11" t="s">
         <v>80</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>24</v>
       </c>
       <c r="J15" s="17">
         <v>45877</v>
@@ -2988,27 +2970,27 @@
         <v>45935</v>
       </c>
       <c r="O15" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P15" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>35</v>
@@ -3020,7 +3002,7 @@
         <v>23</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J16" s="17">
         <v>45877</v>
@@ -3036,27 +3018,27 @@
         <v>45935</v>
       </c>
       <c r="O16" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P16" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F17" s="16" t="s">
         <v>35</v>
@@ -3068,7 +3050,7 @@
         <v>23</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="J17" s="17">
         <v>45877</v>
@@ -3084,10 +3066,10 @@
         <v>45935</v>
       </c>
       <c r="O17" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P17" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -3116,7 +3098,7 @@
         <v>23</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="J18" s="17">
         <v>45877</v>
@@ -3132,39 +3114,39 @@
         <v>45935</v>
       </c>
       <c r="O18" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P18" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="C19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="D19" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="E19" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="E19" s="15" t="s">
-        <v>106</v>
-      </c>
       <c r="F19" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H19" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J19" s="17">
         <v>45877</v>
@@ -3180,27 +3162,27 @@
         <v>45935</v>
       </c>
       <c r="O19" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P19" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="C20" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="15" t="s">
+      <c r="E20" s="15" t="s">
         <v>109</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>110</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>35</v>
@@ -3212,7 +3194,7 @@
         <v>23</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J20" s="17">
         <v>45877</v>
@@ -3232,31 +3214,31 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="C21" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="C21" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="15" t="s">
+      <c r="E21" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="E21" s="15" t="s">
-        <v>115</v>
-      </c>
       <c r="F21" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H21" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J21" s="17">
         <v>45877</v>
@@ -3272,27 +3254,27 @@
         <v>45935</v>
       </c>
       <c r="O21" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P21" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="C22" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D22" s="15" t="s">
+      <c r="E22" s="15" t="s">
         <v>118</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>119</v>
       </c>
       <c r="F22" s="16" t="s">
         <v>35</v>
@@ -3304,7 +3286,7 @@
         <v>23</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J22" s="17">
         <v>45877</v>
@@ -3324,19 +3306,19 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="C23" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="D23" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="E23" s="15" t="s">
         <v>123</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>124</v>
       </c>
       <c r="F23" s="16" t="s">
         <v>35</v>
@@ -3348,7 +3330,7 @@
         <v>23</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J23" s="17">
         <v>45877</v>
@@ -3368,19 +3350,19 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="C24" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="E24" s="15" t="s">
         <v>128</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>129</v>
       </c>
       <c r="F24" s="16" t="s">
         <v>35</v>
@@ -3392,7 +3374,7 @@
         <v>23</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J24" s="17">
         <v>45877</v>
@@ -3412,19 +3394,19 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="C25" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="D25" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="E25" s="15" t="s">
         <v>133</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>134</v>
       </c>
       <c r="F25" s="16" t="s">
         <v>35</v>
@@ -3436,7 +3418,7 @@
         <v>23</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J25" s="17">
         <v>45877</v>
@@ -3456,7 +3438,7 @@
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -3476,31 +3458,31 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="C27" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="D27" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="E27" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="E27" s="15" t="s">
-        <v>140</v>
-      </c>
       <c r="F27" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J27" s="17">
         <v>45877</v>
@@ -3516,39 +3498,39 @@
         <v>45935</v>
       </c>
       <c r="O27" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P27" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="C28" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="D28" s="15" t="s">
+      <c r="E28" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="E28" s="15" t="s">
-        <v>144</v>
-      </c>
       <c r="F28" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H28" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J28" s="17">
         <v>45877</v>
@@ -3564,39 +3546,39 @@
         <v>45935</v>
       </c>
       <c r="O28" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P28" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="C29" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="D29" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="E29" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>149</v>
-      </c>
       <c r="F29" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H29" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J29" s="17">
         <v>45877</v>
@@ -3612,39 +3594,39 @@
         <v>45935</v>
       </c>
       <c r="O29" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P29" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B30" s="15" t="s">
+      <c r="C30" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="D30" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="E30" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="E30" s="15" t="s">
-        <v>154</v>
-      </c>
       <c r="F30" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H30" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J30" s="17">
         <v>45877</v>
@@ -3660,39 +3642,39 @@
         <v>45935</v>
       </c>
       <c r="O30" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P30" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="C31" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="C31" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="D31" s="15" t="s">
+      <c r="E31" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="E31" s="15" t="s">
-        <v>158</v>
-      </c>
       <c r="F31" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J31" s="17">
         <v>45877</v>
@@ -3708,39 +3690,39 @@
         <v>45935</v>
       </c>
       <c r="O31" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P31" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="C32" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="D32" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="E32" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="E32" s="15" t="s">
-        <v>163</v>
-      </c>
       <c r="F32" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H32" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J32" s="17">
         <v>45877</v>
@@ -3756,39 +3738,39 @@
         <v>45935</v>
       </c>
       <c r="O32" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P32" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B33" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="C33" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="D33" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="E33" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="E33" s="15" t="s">
-        <v>168</v>
-      </c>
       <c r="F33" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J33" s="17">
         <v>45877</v>
@@ -3804,27 +3786,27 @@
         <v>45935</v>
       </c>
       <c r="O33" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P33" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="C34" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D34" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="C34" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="D34" s="15" t="s">
+      <c r="E34" s="15" t="s">
         <v>171</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>172</v>
       </c>
       <c r="F34" s="16" t="s">
         <v>35</v>
@@ -3836,7 +3818,7 @@
         <v>23</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>173</v>
+        <v>80</v>
       </c>
       <c r="J34" s="17">
         <v>45877</v>
@@ -3852,27 +3834,27 @@
         <v>45935</v>
       </c>
       <c r="O34" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P34" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D35" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>175</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="E35" s="15" t="s">
-        <v>177</v>
       </c>
       <c r="F35" s="16" t="s">
         <v>35</v>
@@ -3884,7 +3866,7 @@
         <v>23</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>173</v>
+        <v>80</v>
       </c>
       <c r="J35" s="17">
         <v>45877</v>
@@ -3900,27 +3882,27 @@
         <v>45935</v>
       </c>
       <c r="O35" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P35" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="D36" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="E36" s="15" t="s">
         <v>180</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="E36" s="15" t="s">
-        <v>182</v>
       </c>
       <c r="F36" s="16" t="s">
         <v>35</v>
@@ -3932,7 +3914,7 @@
         <v>23</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>173</v>
+        <v>80</v>
       </c>
       <c r="J36" s="17">
         <v>45877</v>
@@ -3948,27 +3930,27 @@
         <v>45935</v>
       </c>
       <c r="O36" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P36" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="D37" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="E37" s="15" t="s">
         <v>185</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="E37" s="15" t="s">
-        <v>187</v>
       </c>
       <c r="F37" s="16" t="s">
         <v>35</v>
@@ -3980,7 +3962,7 @@
         <v>23</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>173</v>
+        <v>80</v>
       </c>
       <c r="J37" s="17">
         <v>45877</v>
@@ -3996,27 +3978,27 @@
         <v>45935</v>
       </c>
       <c r="O37" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P37" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="C38" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="D38" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="E38" s="15" t="s">
         <v>190</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>192</v>
       </c>
       <c r="F38" s="16" t="s">
         <v>35</v>
@@ -4028,7 +4010,7 @@
         <v>23</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J38" s="17">
         <v>45877</v>
@@ -4048,19 +4030,19 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="B39" s="15" t="s">
+      <c r="E39" s="15" t="s">
         <v>195</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="E39" s="15" t="s">
-        <v>197</v>
       </c>
       <c r="F39" s="16" t="s">
         <v>35</v>
@@ -4072,7 +4054,7 @@
         <v>23</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J39" s="17">
         <v>45877</v>
@@ -4092,19 +4074,19 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="C40" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="B40" s="15" t="s">
+      <c r="D40" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="E40" s="15" t="s">
         <v>200</v>
-      </c>
-      <c r="D40" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="E40" s="15" t="s">
-        <v>202</v>
       </c>
       <c r="F40" s="16" t="s">
         <v>35</v>
@@ -4116,7 +4098,7 @@
         <v>23</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J40" s="17">
         <v>45877</v>
@@ -4136,19 +4118,19 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="D41" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="B41" s="15" t="s">
+      <c r="E41" s="15" t="s">
         <v>204</v>
-      </c>
-      <c r="C41" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="D41" s="15" t="s">
-        <v>205</v>
-      </c>
-      <c r="E41" s="15" t="s">
-        <v>206</v>
       </c>
       <c r="F41" s="16" t="s">
         <v>35</v>
@@ -4160,7 +4142,7 @@
         <v>23</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J41" s="17">
         <v>45877</v>
@@ -4180,19 +4162,19 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C42" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="B42" s="15" t="s">
+      <c r="D42" s="15" t="s">
         <v>208</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="E42" s="15" t="s">
         <v>209</v>
-      </c>
-      <c r="D42" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E42" s="15" t="s">
-        <v>211</v>
       </c>
       <c r="F42" s="16" t="s">
         <v>35</v>
@@ -4224,19 +4206,19 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="C43" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="B43" s="15" t="s">
+      <c r="D43" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="C43" s="15" t="s">
+      <c r="E43" s="15" t="s">
         <v>214</v>
-      </c>
-      <c r="D43" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="E43" s="15" t="s">
-        <v>216</v>
       </c>
       <c r="F43" s="16" t="s">
         <v>35</v>
@@ -4268,19 +4250,19 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="D44" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="E44" s="15" t="s">
         <v>218</v>
-      </c>
-      <c r="C44" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="D44" s="15" t="s">
-        <v>219</v>
-      </c>
-      <c r="E44" s="15" t="s">
-        <v>220</v>
       </c>
       <c r="F44" s="16" t="s">
         <v>35</v>
@@ -4312,19 +4294,19 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="D45" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="B45" s="15" t="s">
+      <c r="E45" s="15" t="s">
         <v>222</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="D45" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="E45" s="15" t="s">
-        <v>224</v>
       </c>
       <c r="F45" s="16" t="s">
         <v>35</v>
@@ -4356,7 +4338,7 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -4376,31 +4358,31 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D47" s="15" t="s">
         <v>226</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="E47" s="15" t="s">
         <v>227</v>
       </c>
-      <c r="C47" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="D47" s="15" t="s">
+      <c r="F47" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G47" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="H47" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="I47" s="11" t="s">
         <v>228</v>
-      </c>
-      <c r="E47" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G47" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="H47" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="I47" s="11" t="s">
-        <v>24</v>
       </c>
       <c r="J47" s="17">
         <v>45877</v>
@@ -4416,39 +4398,39 @@
         <v>45935</v>
       </c>
       <c r="O47" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P47" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="B48" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="C48" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="D48" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="D48" s="15" t="s">
+      <c r="E48" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="E48" s="15" t="s">
-        <v>234</v>
-      </c>
       <c r="F48" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H48" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J48" s="17">
         <v>45877</v>
@@ -4464,39 +4446,39 @@
         <v>45935</v>
       </c>
       <c r="O48" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P48" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="C49" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="D49" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="D49" s="15" t="s">
-        <v>238</v>
-      </c>
       <c r="E49" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F49" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H49" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J49" s="17">
         <v>45877</v>
@@ -4512,39 +4494,39 @@
         <v>45935</v>
       </c>
       <c r="O49" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P49" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="B50" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="C50" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="D50" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="E50" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="E50" s="15" t="s">
-        <v>243</v>
-      </c>
       <c r="F50" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G50" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H50" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J50" s="17">
         <v>45877</v>
@@ -4560,39 +4542,39 @@
         <v>45935</v>
       </c>
       <c r="O50" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P50" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B51" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="B51" s="15" t="s">
+      <c r="C51" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="D51" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E51" s="15" t="s">
         <v>246</v>
       </c>
-      <c r="D51" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="E51" s="15" t="s">
-        <v>247</v>
-      </c>
       <c r="F51" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H51" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J51" s="17">
         <v>45877</v>
@@ -4608,39 +4590,39 @@
         <v>45935</v>
       </c>
       <c r="O51" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P51" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="B52" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="B52" s="15" t="s">
+      <c r="C52" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="D52" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="E52" s="15" t="s">
         <v>250</v>
       </c>
-      <c r="D52" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="E52" s="15" t="s">
-        <v>251</v>
-      </c>
       <c r="F52" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G52" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H52" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J52" s="17">
         <v>45877</v>
@@ -4656,27 +4638,27 @@
         <v>45935</v>
       </c>
       <c r="O52" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P52" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B53" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="C53" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="D53" s="15" t="s">
         <v>254</v>
       </c>
-      <c r="D53" s="15" t="s">
+      <c r="E53" s="15" t="s">
         <v>255</v>
-      </c>
-      <c r="E53" s="15" t="s">
-        <v>256</v>
       </c>
       <c r="F53" s="16" t="s">
         <v>35</v>
@@ -4688,7 +4670,7 @@
         <v>23</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J53" s="17">
         <v>45877</v>
@@ -4708,19 +4690,19 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="B54" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="B54" s="15" t="s">
+      <c r="C54" s="15" t="s">
         <v>259</v>
       </c>
-      <c r="C54" s="15" t="s">
+      <c r="D54" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="D54" s="15" t="s">
+      <c r="E54" s="15" t="s">
         <v>261</v>
-      </c>
-      <c r="E54" s="15" t="s">
-        <v>262</v>
       </c>
       <c r="F54" s="16" t="s">
         <v>35</v>
@@ -4732,7 +4714,7 @@
         <v>23</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>263</v>
+        <v>228</v>
       </c>
       <c r="J54" s="17">
         <v>45877</v>
@@ -4748,39 +4730,39 @@
         <v>45935</v>
       </c>
       <c r="O54" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P54" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="C55" s="15" t="s">
         <v>264</v>
       </c>
-      <c r="B55" s="15" t="s">
+      <c r="D55" s="15" t="s">
         <v>265</v>
       </c>
-      <c r="C55" s="15" t="s">
+      <c r="E55" s="15" t="s">
         <v>266</v>
       </c>
-      <c r="D55" s="15" t="s">
-        <v>267</v>
-      </c>
-      <c r="E55" s="15" t="s">
-        <v>268</v>
-      </c>
       <c r="F55" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H55" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J55" s="17">
         <v>45877</v>
@@ -4796,39 +4778,39 @@
         <v>45935</v>
       </c>
       <c r="O55" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P55" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="C56" s="15" t="s">
         <v>269</v>
       </c>
-      <c r="B56" s="15" t="s">
+      <c r="D56" s="15" t="s">
         <v>270</v>
       </c>
-      <c r="C56" s="15" t="s">
+      <c r="E56" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="D56" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="E56" s="15" t="s">
-        <v>273</v>
-      </c>
       <c r="F56" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H56" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="J56" s="17">
         <v>45877</v>
@@ -4844,27 +4826,27 @@
         <v>45935</v>
       </c>
       <c r="O56" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P56" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="D57" s="15" t="s">
         <v>274</v>
       </c>
-      <c r="B57" s="15" t="s">
+      <c r="E57" s="15" t="s">
         <v>275</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>250</v>
-      </c>
-      <c r="D57" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="E57" s="15" t="s">
-        <v>277</v>
       </c>
       <c r="F57" s="16" t="s">
         <v>35</v>
@@ -4876,7 +4858,7 @@
         <v>23</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>278</v>
+        <v>228</v>
       </c>
       <c r="J57" s="17">
         <v>45877</v>
@@ -4892,39 +4874,39 @@
         <v>45935</v>
       </c>
       <c r="O57" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P57" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="B58" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="E58" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="B58" s="15" t="s">
-        <v>280</v>
-      </c>
-      <c r="C58" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="D58" s="15" t="s">
-        <v>281</v>
-      </c>
-      <c r="E58" s="15" t="s">
-        <v>282</v>
-      </c>
       <c r="F58" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G58" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H58" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J58" s="17">
         <v>45877</v>
@@ -4940,39 +4922,39 @@
         <v>45935</v>
       </c>
       <c r="O58" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P58" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="B59" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="D59" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="B59" s="15" t="s">
-        <v>284</v>
-      </c>
-      <c r="C59" s="15" t="s">
-        <v>285</v>
-      </c>
-      <c r="D59" s="15" t="s">
-        <v>286</v>
-      </c>
       <c r="E59" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F59" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H59" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J59" s="17">
         <v>45877</v>
@@ -4988,39 +4970,39 @@
         <v>45935</v>
       </c>
       <c r="O59" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P59" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="B60" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>282</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="E60" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="B60" s="15" t="s">
-        <v>288</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>285</v>
-      </c>
-      <c r="D60" s="15" t="s">
-        <v>289</v>
-      </c>
-      <c r="E60" s="15" t="s">
-        <v>290</v>
-      </c>
       <c r="F60" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G60" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H60" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J60" s="17">
         <v>45877</v>
@@ -5036,39 +5018,39 @@
         <v>45935</v>
       </c>
       <c r="O60" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P60" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E61" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="B61" s="15" t="s">
-        <v>292</v>
-      </c>
-      <c r="C61" s="15" t="s">
-        <v>293</v>
-      </c>
-      <c r="D61" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="E61" s="15" t="s">
-        <v>294</v>
-      </c>
       <c r="F61" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H61" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J61" s="17">
         <v>45877</v>
@@ -5084,39 +5066,39 @@
         <v>45935</v>
       </c>
       <c r="O61" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P61" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F62" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G62" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H62" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J62" s="17">
         <v>45877</v>
@@ -5132,27 +5114,27 @@
         <v>45935</v>
       </c>
       <c r="O62" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P62" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="B63" s="15" t="s">
+        <v>295</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>291</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="E63" s="15" t="s">
         <v>297</v>
-      </c>
-      <c r="B63" s="15" t="s">
-        <v>298</v>
-      </c>
-      <c r="C63" s="15" t="s">
-        <v>294</v>
-      </c>
-      <c r="D63" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="E63" s="15" t="s">
-        <v>300</v>
       </c>
       <c r="F63" s="16" t="s">
         <v>35</v>
@@ -5164,7 +5146,7 @@
         <v>23</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="J63" s="17">
         <v>45877</v>
@@ -5184,7 +5166,7 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="19" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -5212,19 +5194,19 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="D65" s="15" t="s">
         <v>303</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="E65" s="15" t="s">
         <v>304</v>
-      </c>
-      <c r="C65" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="D65" s="15" t="s">
-        <v>306</v>
-      </c>
-      <c r="E65" s="15" t="s">
-        <v>307</v>
       </c>
       <c r="F65" s="16" t="s">
         <v>35</v>
@@ -5236,7 +5218,7 @@
         <v>23</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J65" s="17">
         <v>45877</v>
@@ -5252,27 +5234,27 @@
         <v>45935</v>
       </c>
       <c r="O65" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P65" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="B66" s="15" t="s">
+        <v>306</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>307</v>
+      </c>
+      <c r="D66" s="15" t="s">
+        <v>308</v>
+      </c>
+      <c r="E66" s="15" t="s">
         <v>309</v>
-      </c>
-      <c r="B66" s="15" t="s">
-        <v>310</v>
-      </c>
-      <c r="C66" s="15" t="s">
-        <v>311</v>
-      </c>
-      <c r="D66" s="15" t="s">
-        <v>312</v>
-      </c>
-      <c r="E66" s="15" t="s">
-        <v>313</v>
       </c>
       <c r="F66" s="16" t="s">
         <v>35</v>
@@ -5284,7 +5266,7 @@
         <v>23</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J66" s="17">
         <v>45877</v>
@@ -5304,19 +5286,19 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
+        <v>311</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="D67" s="15" t="s">
+        <v>314</v>
+      </c>
+      <c r="E67" s="15" t="s">
         <v>315</v>
-      </c>
-      <c r="B67" s="15" t="s">
-        <v>316</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>317</v>
-      </c>
-      <c r="D67" s="15" t="s">
-        <v>318</v>
-      </c>
-      <c r="E67" s="15" t="s">
-        <v>319</v>
       </c>
       <c r="F67" s="16" t="s">
         <v>35</v>
@@ -5328,7 +5310,7 @@
         <v>23</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J67" s="17">
         <v>45877</v>
@@ -5344,27 +5326,27 @@
         <v>45935</v>
       </c>
       <c r="O67" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P67" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="B68" s="15" t="s">
+        <v>317</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>319</v>
+      </c>
+      <c r="E68" s="15" t="s">
         <v>320</v>
-      </c>
-      <c r="B68" s="15" t="s">
-        <v>321</v>
-      </c>
-      <c r="C68" s="15" t="s">
-        <v>322</v>
-      </c>
-      <c r="D68" s="15" t="s">
-        <v>323</v>
-      </c>
-      <c r="E68" s="15" t="s">
-        <v>324</v>
       </c>
       <c r="F68" s="16" t="s">
         <v>35</v>
@@ -5376,7 +5358,7 @@
         <v>23</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J68" s="17">
         <v>45877</v>
@@ -5392,27 +5374,27 @@
         <v>45935</v>
       </c>
       <c r="O68" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P68" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="D69" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="E69" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="B69" s="15" t="s">
-        <v>326</v>
-      </c>
-      <c r="C69" s="15" t="s">
-        <v>327</v>
-      </c>
-      <c r="D69" s="15" t="s">
-        <v>328</v>
-      </c>
-      <c r="E69" s="15" t="s">
-        <v>329</v>
       </c>
       <c r="F69" s="16" t="s">
         <v>35</v>
@@ -5424,7 +5406,7 @@
         <v>23</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J69" s="17">
         <v>45877</v>
@@ -5440,27 +5422,27 @@
         <v>45935</v>
       </c>
       <c r="O69" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P69" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="F70" s="16" t="s">
         <v>35</v>
@@ -5472,7 +5454,7 @@
         <v>23</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J70" s="17">
         <v>45877</v>
@@ -5488,27 +5470,27 @@
         <v>45935</v>
       </c>
       <c r="O70" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P70" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="B71" s="15" t="s">
+        <v>331</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>332</v>
+      </c>
+      <c r="D71" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="E71" s="15" t="s">
         <v>334</v>
-      </c>
-      <c r="B71" s="15" t="s">
-        <v>335</v>
-      </c>
-      <c r="C71" s="15" t="s">
-        <v>336</v>
-      </c>
-      <c r="D71" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E71" s="15" t="s">
-        <v>338</v>
       </c>
       <c r="F71" s="16" t="s">
         <v>35</v>
@@ -5520,7 +5502,7 @@
         <v>23</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J71" s="17">
         <v>45877</v>
@@ -5536,27 +5518,27 @@
         <v>45935</v>
       </c>
       <c r="O71" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P71" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
+        <v>335</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="C72" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="D72" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="E72" s="15" t="s">
         <v>339</v>
-      </c>
-      <c r="B72" s="15" t="s">
-        <v>340</v>
-      </c>
-      <c r="C72" s="15" t="s">
-        <v>341</v>
-      </c>
-      <c r="D72" s="15" t="s">
-        <v>342</v>
-      </c>
-      <c r="E72" s="15" t="s">
-        <v>343</v>
       </c>
       <c r="F72" s="16" t="s">
         <v>35</v>
@@ -5568,7 +5550,7 @@
         <v>23</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J72" s="17">
         <v>45877</v>
@@ -5584,27 +5566,27 @@
         <v>45935</v>
       </c>
       <c r="O72" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P72" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>341</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>342</v>
+      </c>
+      <c r="D73" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="E73" s="15" t="s">
         <v>344</v>
-      </c>
-      <c r="B73" s="15" t="s">
-        <v>345</v>
-      </c>
-      <c r="C73" s="15" t="s">
-        <v>346</v>
-      </c>
-      <c r="D73" s="15" t="s">
-        <v>347</v>
-      </c>
-      <c r="E73" s="15" t="s">
-        <v>348</v>
       </c>
       <c r="F73" s="16" t="s">
         <v>35</v>
@@ -5616,7 +5598,7 @@
         <v>23</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J73" s="17">
         <v>45877</v>
@@ -5632,27 +5614,27 @@
         <v>45935</v>
       </c>
       <c r="O73" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P73" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
+        <v>345</v>
+      </c>
+      <c r="B74" s="15" t="s">
+        <v>346</v>
+      </c>
+      <c r="C74" s="15" t="s">
+        <v>347</v>
+      </c>
+      <c r="D74" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="E74" s="15" t="s">
         <v>349</v>
-      </c>
-      <c r="B74" s="15" t="s">
-        <v>350</v>
-      </c>
-      <c r="C74" s="15" t="s">
-        <v>351</v>
-      </c>
-      <c r="D74" s="15" t="s">
-        <v>352</v>
-      </c>
-      <c r="E74" s="15" t="s">
-        <v>353</v>
       </c>
       <c r="F74" s="16" t="s">
         <v>35</v>
@@ -5664,7 +5646,7 @@
         <v>23</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J74" s="17">
         <v>45877</v>
@@ -5680,27 +5662,27 @@
         <v>45935</v>
       </c>
       <c r="O74" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P74" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
+        <v>350</v>
+      </c>
+      <c r="B75" s="15" t="s">
+        <v>351</v>
+      </c>
+      <c r="C75" s="15" t="s">
+        <v>352</v>
+      </c>
+      <c r="D75" s="15" t="s">
+        <v>353</v>
+      </c>
+      <c r="E75" s="15" t="s">
         <v>354</v>
-      </c>
-      <c r="B75" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="C75" s="15" t="s">
-        <v>356</v>
-      </c>
-      <c r="D75" s="15" t="s">
-        <v>357</v>
-      </c>
-      <c r="E75" s="15" t="s">
-        <v>358</v>
       </c>
       <c r="F75" s="16" t="s">
         <v>35</v>
@@ -5712,7 +5694,7 @@
         <v>23</v>
       </c>
       <c r="I75" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J75" s="17">
         <v>45877</v>
@@ -5728,27 +5710,27 @@
         <v>45935</v>
       </c>
       <c r="O75" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P75" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="F76" s="16" t="s">
         <v>35</v>
@@ -5760,7 +5742,7 @@
         <v>23</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J76" s="17">
         <v>45877</v>
@@ -5776,27 +5758,27 @@
         <v>45935</v>
       </c>
       <c r="O76" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P76" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="B77" s="15" t="s">
+        <v>360</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>361</v>
+      </c>
+      <c r="D77" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="E77" s="15" t="s">
         <v>363</v>
-      </c>
-      <c r="B77" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="C77" s="15" t="s">
-        <v>365</v>
-      </c>
-      <c r="D77" s="15" t="s">
-        <v>366</v>
-      </c>
-      <c r="E77" s="15" t="s">
-        <v>367</v>
       </c>
       <c r="F77" s="16" t="s">
         <v>35</v>
@@ -5808,7 +5790,7 @@
         <v>23</v>
       </c>
       <c r="I77" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J77" s="17">
         <v>45877</v>
@@ -5824,27 +5806,27 @@
         <v>45935</v>
       </c>
       <c r="O77" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P77" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
+        <v>364</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>365</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="E78" s="15" t="s">
         <v>368</v>
-      </c>
-      <c r="B78" s="15" t="s">
-        <v>369</v>
-      </c>
-      <c r="C78" s="15" t="s">
-        <v>370</v>
-      </c>
-      <c r="D78" s="15" t="s">
-        <v>371</v>
-      </c>
-      <c r="E78" s="15" t="s">
-        <v>372</v>
       </c>
       <c r="F78" s="16" t="s">
         <v>35</v>
@@ -5856,7 +5838,7 @@
         <v>23</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>308</v>
+        <v>228</v>
       </c>
       <c r="J78" s="17">
         <v>45877</v>
@@ -5872,15 +5854,15 @@
         <v>45935</v>
       </c>
       <c r="O78" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P78" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B79" s="8"/>
       <c r="C79" s="8"/>
@@ -5902,19 +5884,19 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
+        <v>370</v>
+      </c>
+      <c r="B80" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="D80" s="15" t="s">
+        <v>373</v>
+      </c>
+      <c r="E80" s="15" t="s">
         <v>374</v>
-      </c>
-      <c r="B80" s="15" t="s">
-        <v>375</v>
-      </c>
-      <c r="C80" s="15" t="s">
-        <v>376</v>
-      </c>
-      <c r="D80" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="E80" s="15" t="s">
-        <v>378</v>
       </c>
       <c r="F80" s="16" t="s">
         <v>35</v>
@@ -5942,27 +5924,27 @@
         <v>45935</v>
       </c>
       <c r="O80" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P80" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="E81" s="15" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="F81" s="16" t="s">
         <v>35</v>
@@ -5990,39 +5972,39 @@
         <v>45935</v>
       </c>
       <c r="O81" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P81" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>380</v>
+      </c>
+      <c r="C82" s="15" t="s">
+        <v>381</v>
+      </c>
+      <c r="D82" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="E82" s="15" t="s">
         <v>383</v>
       </c>
-      <c r="B82" s="15" t="s">
-        <v>384</v>
-      </c>
-      <c r="C82" s="15" t="s">
-        <v>385</v>
-      </c>
-      <c r="D82" s="15" t="s">
-        <v>386</v>
-      </c>
-      <c r="E82" s="15" t="s">
-        <v>387</v>
-      </c>
       <c r="F82" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G82" s="16" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="H82" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I82" s="11" t="s">
-        <v>388</v>
+        <v>24</v>
       </c>
       <c r="J82" s="17">
         <v>45877</v>
@@ -6038,27 +6020,27 @@
         <v>45935</v>
       </c>
       <c r="O82" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P82" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="22" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="F83" s="16" t="s">
         <v>35</v>
@@ -6086,27 +6068,27 @@
         <v>45935</v>
       </c>
       <c r="O83" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P83" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="22" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="F84" s="16" t="s">
         <v>35</v>
@@ -6134,27 +6116,27 @@
         <v>45935</v>
       </c>
       <c r="O84" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P84" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="F85" s="16" t="s">
         <v>35</v>
@@ -6166,7 +6148,7 @@
         <v>23</v>
       </c>
       <c r="I85" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J85" s="17">
         <v>45877</v>
@@ -6186,19 +6168,19 @@
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="22" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="F86" s="16" t="s">
         <v>35</v>
@@ -6210,7 +6192,7 @@
         <v>23</v>
       </c>
       <c r="I86" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J86" s="17">
         <v>45877</v>
@@ -6230,19 +6212,19 @@
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="22" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="E87" s="15" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="F87" s="16" t="s">
         <v>35</v>
@@ -6254,7 +6236,7 @@
         <v>23</v>
       </c>
       <c r="I87" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J87" s="17">
         <v>45877</v>
@@ -6274,19 +6256,19 @@
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="22" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="E88" s="15" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="F88" s="16" t="s">
         <v>35</v>
@@ -6314,27 +6296,27 @@
         <v>45935</v>
       </c>
       <c r="O88" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P88" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="22" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C89" s="15" t="s">
+        <v>411</v>
+      </c>
+      <c r="D89" s="15" t="s">
         <v>416</v>
       </c>
-      <c r="D89" s="15" t="s">
-        <v>421</v>
-      </c>
       <c r="E89" s="15" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="F89" s="16" t="s">
         <v>35</v>
@@ -6346,7 +6328,7 @@
         <v>23</v>
       </c>
       <c r="I89" s="11" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="J89" s="17">
         <v>45877</v>
@@ -6366,19 +6348,19 @@
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="22" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="E90" s="15" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="F90" s="16" t="s">
         <v>35</v>
@@ -6406,27 +6388,27 @@
         <v>45935</v>
       </c>
       <c r="O90" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P90" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="22" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="E91" s="15" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="F91" s="16" t="s">
         <v>35</v>
@@ -6438,7 +6420,7 @@
         <v>23</v>
       </c>
       <c r="I91" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J91" s="17">
         <v>45877</v>
@@ -6458,19 +6440,19 @@
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="22" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="C92" s="15" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="E92" s="15" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="F92" s="16" t="s">
         <v>35</v>
@@ -6482,7 +6464,7 @@
         <v>23</v>
       </c>
       <c r="I92" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J92" s="17">
         <v>45877</v>
@@ -6502,19 +6484,19 @@
     </row>
     <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="22" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="E93" s="15" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="F93" s="16" t="s">
         <v>35</v>
@@ -6526,7 +6508,7 @@
         <v>23</v>
       </c>
       <c r="I93" s="11" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="J93" s="17">
         <v>45877</v>
@@ -6546,19 +6528,19 @@
     </row>
     <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="22" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="C94" s="15" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="E94" s="15" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="F94" s="16" t="s">
         <v>35</v>
@@ -6570,7 +6552,7 @@
         <v>23</v>
       </c>
       <c r="I94" s="11" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="J94" s="17">
         <v>45877</v>
@@ -6586,15 +6568,15 @@
         <v>45935</v>
       </c>
       <c r="O94" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P94" s="11">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
@@ -6613,31 +6595,31 @@
     </row>
     <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="14" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="E96" s="15" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="F96" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G96" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H96" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I96" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J96" s="17">
         <v>45881</v>
@@ -6653,39 +6635,39 @@
         <v>45987</v>
       </c>
       <c r="O96" s="23">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P96" s="24">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="E97" s="15" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="F97" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H97" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I97" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J97" s="17">
         <v>45881</v>
@@ -6701,39 +6683,39 @@
         <v>45987</v>
       </c>
       <c r="O97" s="23">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P97" s="24">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="14" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="C98" s="15" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="E98" s="15" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="F98" s="16" t="s">
         <v>35</v>
       </c>
       <c r="G98" s="16" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="H98" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I98" s="11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="J98" s="17">
         <v>45881</v>
@@ -6749,27 +6731,27 @@
         <v>45987</v>
       </c>
       <c r="O98" s="23">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P98" s="24">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="C99" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="E99" s="15" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="F99" s="16" t="s">
         <v>35</v>
@@ -6781,7 +6763,7 @@
         <v>23</v>
       </c>
       <c r="I99" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J99" s="17">
         <v>45881</v>
@@ -6800,19 +6782,19 @@
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="B100" s="15" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="C100" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="E100" s="15" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="F100" s="16" t="s">
         <v>35</v>
@@ -6824,7 +6806,7 @@
         <v>23</v>
       </c>
       <c r="I100" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J100" s="17">
         <v>45881</v>
@@ -6843,19 +6825,19 @@
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B101" s="15" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="C101" s="15" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="E101" s="15" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="F101" s="16" t="s">
         <v>35</v>
@@ -6867,7 +6849,7 @@
         <v>23</v>
       </c>
       <c r="I101" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J101" s="17">
         <v>45881</v>
@@ -6886,19 +6868,19 @@
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A102" s="14" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B102" s="15" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="C102" s="15" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="D102" s="15" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="E102" s="15" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="F102" s="16" t="s">
         <v>35</v>
@@ -6910,7 +6892,7 @@
         <v>23</v>
       </c>
       <c r="I102" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J102" s="17">
         <v>45881</v>
@@ -6929,19 +6911,19 @@
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="B103" s="15" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="C103" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="E103" s="15" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="F103" s="16" t="s">
         <v>35</v>
@@ -6953,7 +6935,7 @@
         <v>23</v>
       </c>
       <c r="I103" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J103" s="17">
         <v>45881</v>
@@ -6972,19 +6954,19 @@
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A104" s="14" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="B104" s="15" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="C104" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D104" s="15" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="E104" s="15" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="F104" s="16" t="s">
         <v>35</v>
@@ -6996,7 +6978,7 @@
         <v>23</v>
       </c>
       <c r="I104" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J104" s="17">
         <v>45881</v>
@@ -7015,19 +6997,19 @@
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="B105" s="15" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="C105" s="15" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="E105" s="15" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="F105" s="16" t="s">
         <v>35</v>
@@ -7039,7 +7021,7 @@
         <v>23</v>
       </c>
       <c r="I105" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J105" s="17">
         <v>45881</v>
@@ -7058,19 +7040,19 @@
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A106" s="14" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="B106" s="15" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="C106" s="15" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="E106" s="15" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="F106" s="16" t="s">
         <v>35</v>
@@ -7082,7 +7064,7 @@
         <v>23</v>
       </c>
       <c r="I106" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J106" s="17">
         <v>45881</v>
@@ -7101,19 +7083,19 @@
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="B107" s="15" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="E107" s="15" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="F107" s="16" t="s">
         <v>35</v>
@@ -7125,7 +7107,7 @@
         <v>23</v>
       </c>
       <c r="I107" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J107" s="17">
         <v>45881</v>
@@ -7144,19 +7126,19 @@
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="B108" s="15" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="E108" s="15" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="F108" s="16" t="s">
         <v>35</v>
@@ -7168,7 +7150,7 @@
         <v>23</v>
       </c>
       <c r="I108" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J108" s="17">
         <v>45881</v>
@@ -7187,19 +7169,19 @@
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="B109" s="15" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="E109" s="15" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="F109" s="16" t="s">
         <v>35</v>
@@ -7211,7 +7193,7 @@
         <v>23</v>
       </c>
       <c r="I109" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J109" s="17">
         <v>45881</v>
@@ -7230,19 +7212,19 @@
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A110" s="14" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="B110" s="15" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="E110" s="15" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="F110" s="16" t="s">
         <v>35</v>
@@ -7254,7 +7236,7 @@
         <v>23</v>
       </c>
       <c r="I110" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J110" s="17">
         <v>45881</v>
@@ -7273,19 +7255,19 @@
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A111" s="14" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="B111" s="15" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="E111" s="15" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="F111" s="16" t="s">
         <v>35</v>
@@ -7297,7 +7279,7 @@
         <v>23</v>
       </c>
       <c r="I111" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J111" s="17">
         <v>45881</v>
@@ -7316,19 +7298,19 @@
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A112" s="14" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="E112" s="15" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="F112" s="16" t="s">
         <v>35</v>
@@ -7340,7 +7322,7 @@
         <v>23</v>
       </c>
       <c r="I112" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J112" s="17">
         <v>45881</v>
@@ -7359,19 +7341,19 @@
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113" s="14" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="C113" s="15" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="E113" s="15" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="F113" s="16" t="s">
         <v>35</v>
@@ -7383,7 +7365,7 @@
         <v>23</v>
       </c>
       <c r="I113" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J113" s="17">
         <v>45881</v>
@@ -7402,19 +7384,19 @@
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114" s="14" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="B114" s="15" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="C114" s="15" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D114" s="15" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="E114" s="15" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="F114" s="16" t="s">
         <v>35</v>
@@ -7426,7 +7408,7 @@
         <v>23</v>
       </c>
       <c r="I114" s="11" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J114" s="17">
         <v>45881</v>
@@ -7445,7 +7427,7 @@
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115" s="19" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="B115" s="8"/>
       <c r="C115" s="8"/>
@@ -7472,19 +7454,19 @@
     </row>
     <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="14" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="B116" s="15" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="C116" s="15" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="E116" s="15" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="F116" s="16" t="s">
         <v>35</v>
@@ -7496,7 +7478,7 @@
         <v>23</v>
       </c>
       <c r="I116" s="11" t="s">
-        <v>536</v>
+        <v>80</v>
       </c>
       <c r="J116" s="17">
         <v>45881</v>
@@ -7512,27 +7494,27 @@
         <v>45987</v>
       </c>
       <c r="O116" s="23">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
       <c r="P116" s="24">
-        <v>46191.92044299768</v>
+        <v>46191.95268071759</v>
       </c>
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="B117" s="15" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="E117" s="15" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="F117" s="16" t="s">
         <v>35</v>
@@ -7544,7 +7526,7 @@
         <v>23</v>
       </c>
       <c r="I117" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J117" s="17">
         <v>45881</v>
@@ -7563,19 +7545,19 @@
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="14" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="B118" s="15" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="E118" s="15" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="F118" s="16" t="s">
         <v>35</v>
@@ -7587,7 +7569,7 @@
         <v>23</v>
       </c>
       <c r="I118" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J118" s="17">
         <v>45881</v>
@@ -7606,19 +7588,19 @@
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="B119" s="15" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E119" s="15" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="F119" s="16" t="s">
         <v>35</v>
@@ -7630,7 +7612,7 @@
         <v>23</v>
       </c>
       <c r="I119" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J119" s="17">
         <v>45881</v>
@@ -7649,19 +7631,19 @@
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120" s="14" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="B120" s="15" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="E120" s="15" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="F120" s="16" t="s">
         <v>35</v>
@@ -7673,7 +7655,7 @@
         <v>23</v>
       </c>
       <c r="I120" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J120" s="17">
         <v>45881</v>
@@ -7692,19 +7674,19 @@
     </row>
     <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121" s="14" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="B121" s="15" t="s">
-        <v>556</v>
+        <v>550</v>
       </c>
       <c r="C121" s="15" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="E121" s="15" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="F121" s="16" t="s">
         <v>35</v>
@@ -7716,7 +7698,7 @@
         <v>23</v>
       </c>
       <c r="I121" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J121" s="17">
         <v>45881</v>
@@ -7735,19 +7717,19 @@
     </row>
     <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122" s="14" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="B122" s="15" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="E122" s="15" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="F122" s="16" t="s">
         <v>35</v>
@@ -7759,7 +7741,7 @@
         <v>23</v>
       </c>
       <c r="I122" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J122" s="17">
         <v>45881</v>
@@ -7778,19 +7760,19 @@
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A123" s="14" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="B123" s="15" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E123" s="15" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="F123" s="16" t="s">
         <v>35</v>
@@ -7802,7 +7784,7 @@
         <v>23</v>
       </c>
       <c r="I123" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J123" s="17">
         <v>45881</v>
@@ -7821,19 +7803,19 @@
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A124" s="14" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="B124" s="15" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="C124" s="15" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="E124" s="15" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="F124" s="16" t="s">
         <v>35</v>
@@ -7845,7 +7827,7 @@
         <v>23</v>
       </c>
       <c r="I124" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J124" s="17">
         <v>45881</v>
@@ -7864,19 +7846,19 @@
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A125" s="14" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="B125" s="15" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="E125" s="15" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="F125" s="16" t="s">
         <v>35</v>
@@ -7888,7 +7870,7 @@
         <v>23</v>
       </c>
       <c r="I125" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J125" s="17">
         <v>45881</v>
@@ -7907,19 +7889,19 @@
     </row>
     <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A126" s="14" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="B126" s="15" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="E126" s="15" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="F126" s="16" t="s">
         <v>35</v>
@@ -7931,7 +7913,7 @@
         <v>23</v>
       </c>
       <c r="I126" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J126" s="17">
         <v>45881</v>
@@ -7950,19 +7932,19 @@
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="14" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
       <c r="B127" s="15" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D127" s="15" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="E127" s="15" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="F127" s="16" t="s">
         <v>35</v>
@@ -7974,7 +7956,7 @@
         <v>23</v>
       </c>
       <c r="I127" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J127" s="17">
         <v>45881</v>
@@ -7993,19 +7975,19 @@
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A128" s="14" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="E128" s="15" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="F128" s="16" t="s">
         <v>35</v>
@@ -8017,7 +7999,7 @@
         <v>23</v>
       </c>
       <c r="I128" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J128" s="17">
         <v>45881</v>
@@ -8036,19 +8018,19 @@
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="14" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="B129" s="15" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="C129" s="15" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D129" s="15" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="E129" s="15" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="F129" s="16" t="s">
         <v>35</v>
@@ -8060,7 +8042,7 @@
         <v>23</v>
       </c>
       <c r="I129" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J129" s="17">
         <v>45881</v>
@@ -8079,19 +8061,19 @@
     </row>
     <row r="130" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A130" s="14" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="B130" s="15" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="C130" s="15" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="E130" s="15" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="F130" s="16" t="s">
         <v>35</v>
@@ -8103,7 +8085,7 @@
         <v>23</v>
       </c>
       <c r="I130" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J130" s="17">
         <v>45881</v>
@@ -8122,19 +8104,19 @@
     </row>
     <row r="131" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A131" s="14" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
       <c r="B131" s="15" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="C131" s="15" t="s">
-        <v>593</v>
+        <v>587</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>594</v>
+        <v>588</v>
       </c>
       <c r="E131" s="15" t="s">
-        <v>595</v>
+        <v>589</v>
       </c>
       <c r="F131" s="16" t="s">
         <v>35</v>
@@ -8146,7 +8128,7 @@
         <v>23</v>
       </c>
       <c r="I131" s="11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="J131" s="17">
         <v>45881</v>

</xml_diff>